<commit_message>
criando codigo para coleta de dados do google drive
</commit_message>
<xml_diff>
--- a/empresas.xlsx
+++ b/empresas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,21 +441,1653 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MEDF Serviços Médicos</t>
+          <t>1 - I M PRESTAÇÃO DE SERVIÇOS MÉDICOS LTDA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>49145678000151</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Im49145@2026</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2 - I.A.C.G. PRESTAÇÃO DE SERVIÇOS MÉDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>49456081000128</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>49456081</v>
+      </c>
+      <c r="D3" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3 - MEDF SERVIÇOS MÉDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>49899508000162</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Medf@2025</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>280</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Me49899@2026</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5 - CENTRO TERAPÊUTICO T&amp;T LTDA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>50219602000102</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ded50219@2026</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7 - GASTROMED SERVIÇOS MÉDICOS LTDA.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>51223925000132</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Gastro@2025</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10 - MELISSA XAVIER MENEZES</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>43092673000121</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Melissa@2025</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>11 - PABLO FERNANDES DUARTE MACHADO</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>41933439000154</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Pa41933@2025</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>14 - JM SERVIÇOS MÉDICOS LTDA.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>53206430000120</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Jm53206@2026</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>15 - R. ENERGY REPRESENTAÇÕES LTDA.</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>53967864000143</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Re53967@2026</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>16 - LC SERVICOS DE SAUDE LTDA.</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>54604353000120</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lc54604@2026</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>18 - RRS SAUDE LTDA.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>54650100000192</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Rr54650@2026</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20 - D.A SERVICOS MEDICOS LTDA.</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>54846807000179</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Da54846@2026</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>21 - SOARES E LOBO SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>38826274000107</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Yasmin@2025</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>25 - PSIQUE SERVICOS DE PSICOLOGIA E MEDICINA LTDA</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11314320000132</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Psi11314@2026</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>28 - JP TAMEIRAO GREGORIO SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>55964841000100</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Joao@2025</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>19 - GORDINHO CASTELO COMERCIO DE BEBIDAS LTDA</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>54780099000110</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>123456</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>29 - N MELGACO SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>55954443000103</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nathalia@2025</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>30 - IMPETO LTDA</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>29554530000163</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Im29554@2026</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>31 - RAQUEL ATHAYDE SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>56301185000129</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Raquel@2025</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>32 - VS MEDICINA LTDA</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>56301848000105</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Victor@2025</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>35 - KELEN FERNANDES FISIOTERAPIA LTDA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>57495487000148</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Kelen@2025</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>37 - JCR MEDICINA LTDA</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>57814208000161</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Jc57814@2025</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>38 - FSA SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>55329232000180</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Fs55329@2026</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>39 - MATHEUS EVANGELISTA SIQUEIRA SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>49703898000153</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Matheus@2025</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>40 - IGOR AMARAL SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>53201608000140</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Igor@2025</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>43 - GABRIELLA B SERVICO MEDICO LTDA</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>55769380000115</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Gabriella@2025</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>44 - DMS MEDICINA LTDA</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>59168194000181</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Dm59168@2026</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>45 - GUIMARAES MANGABA INVESTIMENTOS LTDA</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>59120406000150</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Guima59120@2026</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>47 - BRACA SOLUCOES EM EMAGRECIMENTO E TREINAMENTO FISICO LTDA</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>59394664000125</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1vnilGsx</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>48 - NATALIA LOURENCO MESQUITA</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>48939079000147</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>NM48939@2026</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>49 - BRUNA PB SERVICOS EM FISIOTERAPIA LIMITADA</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>55989486000124</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Bruna@2025</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>50 - ANA GABRIELA ANDRADE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>46052636000188</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Ana46052@2026</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>51 - GABRIELA AMORIM DE CASTRO</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>42350638000100</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Gab42350@2026</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>52 - ENFANT CLINICA PEDIATRICA LTDA</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>45838235000195</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Enfant@2025</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>54 - SOLLON NATHAN FREITAS ALMEIDA SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>58435946000160</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>49456081</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>56 - DG PALESTRAS E SAUDE LTDA</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>60287845000131</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Dg60287@2026</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>57 - BRAGA SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>48813080000120</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Braga@2025</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>58 - MAIPO SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>61030387000113</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Maipo@2025</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>59 - THAIS QUARESMA MEDICINA LTDA</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>61257595000150</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Thais@2025</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>61 - GUILHERME DUTRA SAUDE LTDA</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>61869250000157</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Guilherme@2025</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>62 - JOYCE RODRIGUES SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>62219409000150</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Joyce@2025</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>63 - MACIEL SERVICO MEDICO LTDA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>62350101000140</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Yasmin@2025</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>64 - LNAS SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>62412593000150</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Livia@2025</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>65 - JULIA RAYANE FERREIRA SILVA LTDA</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>55571256000140</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1234567@</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>66 - MARCELA SILVA NASCIMENTO</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>62781581000101</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Marcela@2025</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>67 - N.X. SERVICOS MEDICOS LTDA.</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>63167240000103</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Marina@2025</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>68 - INSTITUTO SYNAPSE LTDA</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>63155137000135</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Synapse@2025</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>69 - FB SERVICOS VETERINARIOS LTDA.</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>63289874000120</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Fernanda@2025</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>70 - LLN SERVICOS ADMINISTRATIVOS E TREINAMENTOS LTDA</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>63391724000123</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Lln@2025</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>71 - ONSTAGE SOLUÇÕES FINANCEIRAS LTDA</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>48744243000160</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Onstage@2026</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>73 - NJ RESENDE SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>53364064000138</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>NjMed@2025</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>74 - DB AVIATION LTDA</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>63415967000154</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Diego@2025</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>75 - GRC MEDICINA LTDA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>63597425000140</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Gr63597@2025</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>76 - RAQUIMA SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>63747193000169</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Ra63747@2025</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>77 - BENESSERE SERVICOS MEDICOS LTDA.</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>63777158000192</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Be63777@2025</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>78 - CARDIOVET SERVICOS VETERINARIOS LTDA</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>63820094000165</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Be63777@2025</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>79 - MJCJR SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>63838084000157</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Ab63838@2025</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>81 - ALTOMARE OFTALMOLOGIA VETERINARIA LTDA</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>63920962000189</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Al63920@2026</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>82 - ALF SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>64071221000133</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Al64071@2026</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>83 - VSENRA SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>64160854000118</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Se64160@2026</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>84 - MV. MATHEUS ANTONIO SERVICOS VETERINARIOS LTDA</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>64161062000168</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Ma64161@2025</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>85 - MQ SERVICOS MEDICOS VETERINARIOS LTDA</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>64161199000112</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>So64161@2026</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>86 - LG VET SERVICOS MEDICOS VETERINARIOS LTDA</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>64166285000118</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Lg64166@2026</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>87 - TOITIO SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>64126604000161</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Gabriela2026</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>88 - AJPS SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>64302917000123</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Al64302@2026</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>89 - JULIA PRADO POUZAS SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>64336739000151</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Pr64336@2026</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>90 - JVO SERVICOS MEDICOS LTDA.</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>64352827000147</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Jo64352@2026</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>91 - GONCALOS GUIMARAES SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>64358418000158</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>IG64358@2026</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>92 - MLJ SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>64380278000114</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Ml64380@2026</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>93 - AJT SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>64417135000130</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Aj64417@2026</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>94 - AHOC SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>64613401000108</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Ah64613@2026</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>95 - RAFAELLA OLIVEIRA NEUROLOGIA VETERINARIA LTDA</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>24898695000139</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Ra24898@2026</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>96 - IVK PRESTACAO DE SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>56703029000194</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>JHZ3duue</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>97 - 50.666.021 MILENA MARIA FERREIRA DE PAULA</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>50666021000119</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Mi50666@2026</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>98 - BRUNO VALADARES PEREIRA SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>57431668000100</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Br57431@2026</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>99 - LARISSA SANTIAGO GASTROENTEROLOGIA E HEPATOLOGIA VETERINARIA LTDA</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>64944773000109</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>La64944@2026</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>100 - ISABELLA OLIVEIRA RODARTE SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>61487677000190</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>1234</v>
+      </c>
+      <c r="D78" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>101 - ALMEIDA &amp; SANTOS SERVICOS DE PRESTACOES HOSPITALARES LTDA</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>61939964000194</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ma32548017</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>102 - DERMAPET AC VETERINARIA LTDA</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>65018703000192</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>De65018@2026</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>103 - M. LOPES SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>65088161000124</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Medicina07!</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>104 - GASPAR SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>65736857000110</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Ga65736@2026</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>105 - RIBEIRO NUNES SERVICOS MEDICOS LTDA.</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>65859239000167</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Rib65859@2026</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>106 - DH SERVICOS MEDICOS LTDA</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>65866405000152</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Si65866@2026</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>